<commit_message>
Lots of data updates
</commit_message>
<xml_diff>
--- a/IndirectBP/OverallStatsIndirectBP-noboot.xlsx
+++ b/IndirectBP/OverallStatsIndirectBP-noboot.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexb\OneDrive\Documents\Thesis\IndirectBP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC8AC242-BF27-4E8E-B0F7-5C4E8CDC3BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A870CDE8-A04D-4C4B-860B-BEE4FA21F27F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{84A3B88E-B226-40B3-A64E-0FDCC502A4B5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{84A3B88E-B226-40B3-A64E-0FDCC502A4B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>HalfCache</t>
   </si>
@@ -74,9 +74,6 @@
     <t>Swaptions</t>
   </si>
   <si>
-    <t>Nu: 0.0001, Gamma: 0.0001</t>
-  </si>
-  <si>
     <t>Vips</t>
   </si>
   <si>
@@ -116,16 +113,31 @@
     <t>Specificity</t>
   </si>
   <si>
-    <t>Nu: 0.9, Gamma: 0.2</t>
-  </si>
-  <si>
     <t>NU and Gamma</t>
   </si>
   <si>
     <t>Dedup</t>
   </si>
   <si>
-    <t>Nu: 0.2, Gamma: 0.7</t>
+    <t>Nu: 0.9, Gamma: 0.0625</t>
+  </si>
+  <si>
+    <t>Nu: 0.99, Gamma: 0.0625</t>
+  </si>
+  <si>
+    <t>Nu: 0.7, Gamma: 0.0001</t>
+  </si>
+  <si>
+    <t>Nu: 0.1, Gamma: 0.7</t>
+  </si>
+  <si>
+    <t>Nu: 0.0002, Gamma: 0.99</t>
+  </si>
+  <si>
+    <t>Nu: 0.7, Gamma: 0.99</t>
+  </si>
+  <si>
+    <t>Nu: 0.99, Gamma: 0.2</t>
   </si>
 </sst>
 </file>
@@ -498,66 +510,66 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{652EE7E4-9A64-4328-97BF-22E9AA604A6A}">
   <dimension ref="A1:M14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.36328125" customWidth="1"/>
+    <col min="1" max="1" width="34.33203125" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
-    <col min="7" max="7" width="22.26953125" customWidth="1"/>
-    <col min="11" max="11" width="14.7265625" customWidth="1"/>
+    <col min="7" max="7" width="22.21875" customWidth="1"/>
+    <col min="11" max="11" width="14.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
         <v>15</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" t="s">
-        <v>24</v>
-      </c>
-      <c r="K2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>20</v>
       </c>
-      <c r="M2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -569,7 +581,7 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G3">
         <v>100</v>
@@ -597,7 +609,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -614,26 +626,26 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G4">
-        <v>97.674418599999996</v>
+        <v>97.619047620000003</v>
       </c>
       <c r="H4">
-        <f t="shared" ref="H4:H13" si="0">(C4)/(C4+D4)</f>
+        <f t="shared" ref="H4:H7" si="0">(C4)/(C4+D4)</f>
         <v>0.75</v>
       </c>
       <c r="I4">
-        <f t="shared" ref="I4:I13" si="1">C4/(C4+E4)</f>
+        <f t="shared" ref="I4" si="1">C4/(C4+E4)</f>
         <v>1</v>
       </c>
       <c r="J4">
-        <f t="shared" ref="J4:J13" si="2">(2*(H4*I4))/(H4+I4)</f>
+        <f t="shared" ref="J4:J6" si="2">(2*(H4*I4))/(H4+I4)</f>
         <v>0.8571428571428571</v>
       </c>
       <c r="K4">
-        <f t="shared" ref="K4:K13" si="3">F4/(F4+D4)</f>
-        <v>0.97499999999999998</v>
+        <f t="shared" ref="K4:K6" si="3">F4/(F4+D4)</f>
+        <v>0.97435897435897434</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -642,43 +654,43 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G5">
-        <v>89.090909089999997</v>
+        <v>92.452830188679201</v>
       </c>
       <c r="H5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I5" t="e">
+        <v>0.2</v>
+      </c>
+      <c r="I5">
         <f>C5/(C5+E5)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J5" t="e">
+        <v>1</v>
+      </c>
+      <c r="J5">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>0.33333333333333337</v>
       </c>
       <c r="K5">
         <f t="shared" si="3"/>
-        <v>0.89090909090909087</v>
+        <v>0.92307692307692313</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -687,60 +699,60 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D6">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F6">
-        <v>2746</v>
+        <v>2727</v>
       </c>
       <c r="G6">
-        <v>99.637155300000003</v>
+        <v>99.128856619999993</v>
       </c>
       <c r="H6">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I6" t="e">
+        <v>0.4</v>
+      </c>
+      <c r="I6">
         <f t="shared" ref="I6:I7" si="4">C6/(C6+E6)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J6" t="e">
+        <v>0.18181818181818182</v>
+      </c>
+      <c r="J6">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>0.25000000000000006</v>
       </c>
       <c r="K6">
         <f t="shared" si="3"/>
-        <v>0.99637155297532654</v>
+        <v>0.99780461031833145</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M6">
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -749,98 +761,170 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="G7">
-        <v>99.901088031651796</v>
+        <v>99.900891972249696</v>
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
-        <v>0.95833333333333337</v>
+        <v>0.95652173913043481</v>
       </c>
       <c r="I7">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="J7">
-        <f t="shared" ref="J7:J14" si="5">(2*(H7*I7))/(H7+I7)</f>
-        <v>0.97872340425531912</v>
+        <f t="shared" ref="J7:J9" si="5">(2*(H7*I7))/(H7+I7)</f>
+        <v>0.97777777777777775</v>
       </c>
       <c r="K7">
         <f t="shared" ref="K7:K14" si="6">F7/(F7+D7)</f>
-        <v>0.99898785425101211</v>
+        <v>0.99898682877406286</v>
       </c>
       <c r="L7">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M7">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="H8" t="e">
-        <f t="shared" ref="H7:H14" si="7">(C8)/(C8+D8)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I8" t="e">
-        <f t="shared" ref="I7:I14" si="8">C8/(C8+E8)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J8" t="e">
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>118</v>
+      </c>
+      <c r="G8">
+        <v>97.540983606557305</v>
+      </c>
+      <c r="H8">
+        <f t="shared" ref="H8:H14" si="7">(C8)/(C8+D8)</f>
+        <v>0.25</v>
+      </c>
+      <c r="I8">
+        <f t="shared" ref="I8:I9" si="8">C8/(C8+E8)</f>
+        <v>1</v>
+      </c>
+      <c r="J8">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K8" t="e">
+        <v>0.4</v>
+      </c>
+      <c r="K8">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+        <v>0.97520661157024791</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="H9" t="e">
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9">
+        <v>4</v>
+      </c>
+      <c r="F9">
+        <v>182</v>
+      </c>
+      <c r="G9">
+        <v>94.059405940594004</v>
+      </c>
+      <c r="H9">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I9" t="e">
+        <v>0.5</v>
+      </c>
+      <c r="I9">
         <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J9" t="e">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="J9">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K9" t="e">
+        <v>0.57142857142857151</v>
+      </c>
+      <c r="K9">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+        <v>0.95789473684210524</v>
+      </c>
+      <c r="L9">
+        <v>10</v>
+      </c>
+      <c r="M9">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="H10" t="e">
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>32</v>
+      </c>
+      <c r="G10">
+        <v>94.285714285714207</v>
+      </c>
+      <c r="H10">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I10" t="e">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="I10">
         <f>C10/(C10+E10)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J10" t="e">
+        <v>1</v>
+      </c>
+      <c r="J10">
         <f>(2*(H10*I10))/(H10+I10)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K10" t="e">
+        <v>0.5</v>
+      </c>
+      <c r="K10">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+        <v>0.94117647058823528</v>
+      </c>
+      <c r="L10">
+        <v>10</v>
+      </c>
+      <c r="M10">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -861,7 +945,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -882,9 +966,9 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H13" t="e">
         <f t="shared" si="7"/>
@@ -903,25 +987,49 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" t="e">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14">
+        <v>144</v>
+      </c>
+      <c r="D14">
+        <v>358</v>
+      </c>
+      <c r="E14">
+        <v>69</v>
+      </c>
+      <c r="F14">
+        <v>4948</v>
+      </c>
+      <c r="G14">
+        <v>92.26309114</v>
+      </c>
+      <c r="H14">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I14" t="e">
+        <v>0.28685258964143429</v>
+      </c>
+      <c r="I14">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J14" t="e">
+        <v>0.676056338028169</v>
+      </c>
+      <c r="J14">
         <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K14" t="e">
+        <v>0.40279720279720288</v>
+      </c>
+      <c r="K14">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>0.93252921221258955</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finished Analysis for IndirectBP
</commit_message>
<xml_diff>
--- a/IndirectBP/OverallStatsIndirectBP-noboot.xlsx
+++ b/IndirectBP/OverallStatsIndirectBP-noboot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexb\OneDrive\Documents\Thesis\IndirectBP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A870CDE8-A04D-4C4B-860B-BEE4FA21F27F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{445C066D-5F98-41AA-B65C-54CACFF3A4E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{84A3B88E-B226-40B3-A64E-0FDCC502A4B5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t>HalfCache</t>
   </si>
@@ -138,6 +138,15 @@
   </si>
   <si>
     <t>Nu: 0.99, Gamma: 0.2</t>
+  </si>
+  <si>
+    <t>Nu: 0.2, Gamma: 0.9</t>
+  </si>
+  <si>
+    <t>Nu: 0.5, Gamma: 0.5</t>
+  </si>
+  <si>
+    <t>Nu: 0.9, Gamma: 0.5</t>
   </si>
 </sst>
 </file>
@@ -928,63 +937,135 @@
       <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="H11" t="e">
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11">
+        <v>9</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>240</v>
+      </c>
+      <c r="G11">
+        <v>98.809523809523796</v>
+      </c>
+      <c r="H11">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I11" t="e">
+        <v>0.75</v>
+      </c>
+      <c r="I11">
         <f t="shared" ref="I11:I14" si="9">C11/(C11+E11)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J11" t="e">
+        <v>1</v>
+      </c>
+      <c r="J11">
         <f t="shared" ref="J11:J14" si="10">(2*(H11*I11))/(H11+I11)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K11" t="e">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="K11">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>0.98765432098765427</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="H12" t="e">
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>2</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>30</v>
+      </c>
+      <c r="G12">
+        <v>94.285714285714207</v>
+      </c>
+      <c r="H12">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I12" t="e">
+        <v>0.6</v>
+      </c>
+      <c r="I12">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J12" t="e">
+        <v>1</v>
+      </c>
+      <c r="J12">
         <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K12" t="e">
+        <v>0.74999999999999989</v>
+      </c>
+      <c r="K12">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>0.9375</v>
+      </c>
+      <c r="L12">
+        <v>10</v>
+      </c>
+      <c r="M12">
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="H13" t="e">
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>10</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>113</v>
+      </c>
+      <c r="G13">
+        <v>92</v>
+      </c>
+      <c r="H13">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I13" t="e">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="I13">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J13" t="e">
+        <v>1</v>
+      </c>
+      <c r="J13">
         <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K13" t="e">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="K13">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>0.91869918699186992</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>